<commit_message>
Auto-persist dialogue artifacts and delta_scraper refinements
</commit_message>
<xml_diff>
--- a/MACCRE_Global.xlsx
+++ b/MACCRE_Global.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,12 +99,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00888888"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00276221"/>
       <sz val="10"/>
@@ -116,7 +110,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -151,11 +145,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F0F0F8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8F9FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -195,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -225,15 +214,14 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -599,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -832,152 +820,159 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>gemini-embedding-001</t>
+          <t>gemini-3.5-live-translate-preview</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>gemini-embedding-2</t>
+          <t>gemini-embedding-001</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>gemini-embedding-2-preview</t>
+          <t>gemini-embedding-2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>gemini-flash-latest</t>
+          <t>gemini-embedding-2-preview</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>gemini-flash-lite-latest</t>
+          <t>gemini-flash-latest</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>gemini-pro-latest</t>
+          <t>gemini-flash-lite-latest</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>gemini-robotics-er-1.5-preview</t>
+          <t>gemini-pro-latest</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>gemini-robotics-er-1.6-preview</t>
+          <t>gemini-robotics-er-1.5-preview</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>gemma-4-26b-a4b-it</t>
+          <t>gemini-robotics-er-1.6-preview</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>gemma-4-31b-it</t>
+          <t>gemma-4-26b-a4b-it</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>imagen-4.0-fast-generate-001</t>
+          <t>gemma-4-31b-it</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>imagen-4.0-generate-001</t>
+          <t>imagen-4.0-fast-generate-001</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>imagen-4.0-ultra-generate-001</t>
+          <t>imagen-4.0-generate-001</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>lyria-3-clip-preview</t>
+          <t>imagen-4.0-ultra-generate-001</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>lyria-3-pro-preview</t>
+          <t>lyria-3-clip-preview</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>nano-banana-pro-preview</t>
+          <t>lyria-3-pro-preview</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>veo-2.0-generate-001</t>
+          <t>nano-banana-pro-preview</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>veo-3.0-fast-generate-001</t>
+          <t>veo-2.0-generate-001</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>veo-3.0-generate-001</t>
+          <t>veo-3.0-fast-generate-001</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>veo-3.1-fast-generate-preview</t>
+          <t>veo-3.0-generate-001</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>veo-3.1-generate-preview</t>
+          <t>veo-3.1-fast-generate-preview</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
+        <is>
+          <t>veo-3.1-generate-preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>veo-3.1-lite-generate-preview</t>
         </is>
@@ -1203,7 +1198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1256,6 +1251,64 @@
       <c r="G2" s="6" t="inlineStr">
         <is>
           <t>CREATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>20260609-221021-5tcw</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>META_TEST</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr"/>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="n">
+        <v>0.0234</v>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09 22:10:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>20260609-220935-oh89</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>META_TEST</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr"/>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>0.0234</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09 22:09:35</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1333,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>◈  MACCRE_GLOBAL.xlsx — Quick Reference  ◈</t>
         </is>
@@ -1937,12 +1990,195 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>[EXO_TEST] OSINT_Analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[EXO_TEST] Regular_Joe</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>[EXO_TEST] CounterPartner</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>[EXO_TEST] TopperShepherd</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>[EXO_TEST] TopperAngry</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>[EXO_TEST] TopperBuddy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>[EXO_TEST] GretchenHarwell</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>[MEMORY_TEST] MemoryReporter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>[META_TEST] MemoryReporter</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>[META_TEST] SourceReader</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>[META_TEST] Synthesizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[T1_SMOKE] TestAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>[T2_FAILURE] TestAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>[T3_DIAMOND] TestAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>[T4_RACE] TestAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>[T4_RACE] DetailAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>[T5_LOOP] TestAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>[T5_LOOP] JudgeAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>[T6_VALIDATE] TestAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>[T7_DIALOGUE] TestAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>[T7_DIALOGUE] AnalystAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>[T7_DIALOGUE] SkepticAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>[T8_GROUP_DIALOGUE] TestAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>[T8_GROUP_DIALOGUE] HostAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>[T8_GROUP_DIALOGUE] OptimistAgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>[T8_GROUP_DIALOGUE] PessimistAgent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2001,7 +2237,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>META_TEST</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -2075,6 +2311,11 @@
       <c r="A7" s="1" t="inlineStr">
         <is>
           <t>LINKED_PROJECTS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MEMORY_TEST</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -2231,7 +2472,7 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="New Project?" error="This name is not in the existing project list. Continue to auto-provision a new project silo." type="list" errorStyle="warning">
-      <formula1>"GLOBAL"</formula1>
+      <formula1>"GLOBAL,MEMORY_TEST,EXO_TEST"</formula1>
     </dataValidation>
     <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Choose a value from the dropdown list." type="list" errorStyle="stop">
       <formula1>"TRUE,FALSE"</formula1>
@@ -2354,634 +2595,454 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>MyAgent</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>gemini-2.5-flash</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MemoryReporter</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>Researcher</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>You are MyAgent, a precise research agent...</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>search_web|write_file</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr"/>
-      <c r="H3" s="13" t="inlineStr"/>
-      <c r="I3" s="13" t="inlineStr"/>
-      <c r="J3" s="13" t="inlineStr"/>
-      <c r="K3" s="13" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>You are the MemoryReporter. Your task is to query the MEMORY_TEST project database. First, call import_foreign_vectors('MEMORY_TEST', 2.0). Then, use iterative_scoped_search to discover concepts from MEMORY_TEST. Present a detailed summary of these past memories to the group.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>import_foreign_vectors|iterative_scoped_search</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>Local Only</t>
         </is>
       </c>
-      <c r="L3" s="13" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="M3" s="13" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="N3" s="13" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>cloud</t>
         </is>
       </c>
       <c r="O3" s="7" t="n"/>
-      <c r="P3" s="9" t="inlineStr"/>
+      <c r="P3" s="9" t="n"/>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SourceReader</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>You are the SourceReader. Your task is to read the raw source documents for this project. Use read_file to read the following 4 files in the 01_Raw_Source directory: AIethics.md, HolographicInterferometry.md, LlamdaLlamdaLlamda.md, SentinelOSarch.md. Summarise their contents and present your findings to the group.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>read_file</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Local Only</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>cloud</t>
+        </is>
+      </c>
       <c r="O4" s="7" t="n"/>
-      <c r="P4" s="10" t="inlineStr">
-        <is>
-          <t>ROLES  (col C)  — Diamond Loop position</t>
-        </is>
-      </c>
+      <c r="P4" s="10" t="n"/>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Synthesizer</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Synthesiser</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>You are the Synthesizer. Read the chat history carefully to ingest the reports from the MemoryReporter and the SourceReader. Combine their insights into a single cohesive artifact that connects the historical memory with the new source documents. Write your final report to 04_Code_Artifacts/final_synthesis.md using the write_file tool.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>write_file</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Local Only</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>cloud</t>
+        </is>
+      </c>
       <c r="O5" s="7" t="n"/>
-      <c r="P5" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Researcher   temp 1.0  Early pipeline. Data gathering.</t>
-        </is>
-      </c>
+      <c r="P5" s="11" t="n"/>
     </row>
     <row r="6">
       <c r="O6" s="7" t="n"/>
-      <c r="P6" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Writer       temp 1.0  Content generation.</t>
-        </is>
-      </c>
+      <c r="P6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="O7" s="7" t="n"/>
-      <c r="P7" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Synthesiser  temp 1.0  Fan-in merge. Use with WAIT_FOR.</t>
-        </is>
-      </c>
+      <c r="P7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="O8" s="7" t="n"/>
-      <c r="P8" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Director     temp 1.0  Orchestration and routing logic.</t>
-        </is>
-      </c>
+      <c r="P8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="O9" s="7" t="n"/>
-      <c r="P9" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Critic       temp 0.1  Quality gate. Loops w/ MAX_REC.</t>
-        </is>
-      </c>
+      <c r="P9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="O10" s="7" t="n"/>
-      <c r="P10" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Extractor    temp 0.1  Structured output. json required.</t>
-        </is>
-      </c>
+      <c r="P10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="O11" s="7" t="n"/>
-      <c r="P11" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Verifier     temp 0.1  OSINT epistemic gate. Pre-render.</t>
-        </is>
-      </c>
+      <c r="P11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="O12" s="7" t="n"/>
-      <c r="P12" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Renderer     temp 0.1  Fires A/V pipeline. Terminal.</t>
-        </is>
-      </c>
+      <c r="P12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="O13" s="7" t="n"/>
-      <c r="P13" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Archivist    temp 0.1  Writes to knowledge store.</t>
-        </is>
-      </c>
+      <c r="P13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="O14" s="7" t="n"/>
-      <c r="P14" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Router       temp 1.0  Pure routing. Minimal generation.</t>
-        </is>
-      </c>
+      <c r="P14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="O15" s="7" t="n"/>
-      <c r="P15" s="9" t="inlineStr"/>
+      <c r="P15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="O16" s="7" t="n"/>
-      <c r="P16" s="10" t="inlineStr">
-        <is>
-          <t>SEARCH_GROUNDING  (col K)</t>
-        </is>
-      </c>
+      <c r="P16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="O17" s="7" t="n"/>
-      <c r="P17" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Local Only        Thought pins → vector query. Default.</t>
-        </is>
-      </c>
+      <c r="P17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="O18" s="7" t="n"/>
-      <c r="P18" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Google            Gemini native search grounding.</t>
-        </is>
-      </c>
+      <c r="P18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="O19" s="7" t="n"/>
-      <c r="P19" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Brave             Brave Search API. Add search_web tool.</t>
-        </is>
-      </c>
+      <c r="P19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="O20" s="7" t="n"/>
-      <c r="P20" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Hybrid            Google feeds Brave sequentially.</t>
-        </is>
-      </c>
+      <c r="P20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="O21" s="7" t="n"/>
-      <c r="P21" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Hybrid-Synthesis  Parallel G+B → dedup → labelled list.</t>
-        </is>
-      </c>
+      <c r="P21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="O22" s="7" t="n"/>
-      <c r="P22" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Hybrid-Synthesis: use execute_hybrid_synthesis tool.</t>
-        </is>
-      </c>
+      <c r="P22" s="12" t="n"/>
     </row>
     <row r="23">
       <c r="O23" s="7" t="n"/>
-      <c r="P23" s="9" t="inlineStr"/>
+      <c r="P23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="O24" s="7" t="n"/>
-      <c r="P24" s="10" t="inlineStr">
-        <is>
-          <t>RESPONSE_FORMAT  (col L)</t>
-        </is>
-      </c>
+      <c r="P24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="O25" s="7" t="n"/>
-      <c r="P25" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  markdown  Prose output. Default for generators.</t>
-        </is>
-      </c>
+      <c r="P25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="O26" s="7" t="n"/>
-      <c r="P26" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  json      API-enforced. Required: Extractor / Critic.</t>
-        </is>
-      </c>
+      <c r="P26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="O27" s="7" t="n"/>
-      <c r="P27" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  text      Plain text, no formatting.</t>
-        </is>
-      </c>
+      <c r="P27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="O28" s="7" t="n"/>
-      <c r="P28" s="9" t="inlineStr"/>
+      <c r="P28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="O29" s="7" t="n"/>
-      <c r="P29" s="10" t="inlineStr">
-        <is>
-          <t>TEMPERATURE — Diamond Loop Doctrine</t>
-        </is>
-      </c>
+      <c r="P29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="O30" s="7" t="n"/>
-      <c r="P30" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1.0  Generators: Researcher, Writer, Director</t>
-        </is>
-      </c>
+      <c r="P30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="O31" s="7" t="n"/>
-      <c r="P31" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.1  Critics:    Extractor, Critic, Verifier</t>
-        </is>
-      </c>
+      <c r="P31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="O32" s="7" t="n"/>
-      <c r="P32" s="9" t="inlineStr"/>
+      <c r="P32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="O33" s="7" t="n"/>
-      <c r="P33" s="10" t="inlineStr">
-        <is>
-          <t>TOOLS  (col F) — pipe-separated, e.g. search_web|write_file</t>
-        </is>
-      </c>
+      <c r="P33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="O34" s="7" t="n"/>
-      <c r="P34" s="9" t="inlineStr"/>
+      <c r="P34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="O35" s="7" t="n"/>
-      <c r="P35" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Web &amp; OSINT</t>
-        </is>
-      </c>
+      <c r="P35" s="10" t="n"/>
     </row>
     <row r="36">
       <c r="O36" s="7" t="n"/>
-      <c r="P36" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  search_web               Brave Search API</t>
-        </is>
-      </c>
+      <c r="P36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="O37" s="7" t="n"/>
-      <c r="P37" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  read_url_content          Fetch + parse a URL</t>
-        </is>
-      </c>
+      <c r="P37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="O38" s="7" t="n"/>
-      <c r="P38" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  execute_hybrid_synthesis  G+B parallel dedup search</t>
-        </is>
-      </c>
+      <c r="P38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="O39" s="7" t="n"/>
-      <c r="P39" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Memory &amp; RAG</t>
-        </is>
-      </c>
+      <c r="P39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="O40" s="7" t="n"/>
-      <c r="P40" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  query_local_memory        Vector search in project silo</t>
-        </is>
-      </c>
+      <c r="P40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="O41" s="7" t="n"/>
-      <c r="P41" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  fts_search_memory         BM25 full-text search</t>
-        </is>
-      </c>
+      <c r="P41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="O42" s="7" t="n"/>
-      <c r="P42" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ingest_document           Hash-aware doc ingest</t>
-        </is>
-      </c>
+      <c r="P42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="O43" s="7" t="n"/>
-      <c r="P43" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  query_foreign_memory      Search linked project silo</t>
-        </is>
-      </c>
+      <c r="P43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="O44" s="7" t="n"/>
-      <c r="P44" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  import_foreign_vectors    Pull vectors from linked silo</t>
-        </is>
-      </c>
+      <c r="P44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="O45" s="7" t="n"/>
-      <c r="P45" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  prune_semantic_memory     Remove stale embeddings</t>
-        </is>
-      </c>
+      <c r="P45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="O46" s="7" t="n"/>
-      <c r="P46" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  File I/O</t>
-        </is>
-      </c>
+      <c r="P46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="O47" s="7" t="n"/>
-      <c r="P47" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  read_file                 Read from DATACENTER</t>
-        </is>
-      </c>
+      <c r="P47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="O48" s="7" t="n"/>
-      <c r="P48" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  write_file                Write to 04_ or 05_ tier</t>
-        </is>
-      </c>
+      <c r="P48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="O49" s="7" t="n"/>
-      <c r="P49" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  file_exists               Check DATACENTER path</t>
-        </is>
-      </c>
+      <c r="P49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="O50" s="7" t="n"/>
-      <c r="P50" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  trash_file                Move file to trash (needs elevation)</t>
-        </is>
-      </c>
+      <c r="P50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="O51" s="7" t="n"/>
-      <c r="P51" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Telemetry</t>
-        </is>
-      </c>
+      <c r="P51" s="10" t="n"/>
     </row>
     <row r="52">
       <c r="O52" s="7" t="n"/>
-      <c r="P52" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  query_thoughts            Read L1 session thoughts</t>
-        </is>
-      </c>
+      <c r="P52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="O53" s="7" t="n"/>
-      <c r="P53" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  query_telemetry_matrix    Query cost + event data</t>
-        </is>
-      </c>
+      <c r="P53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="O54" s="7" t="n"/>
-      <c r="P54" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  read_local_codebase       Self-audit Python source</t>
-        </is>
-      </c>
+      <c r="P54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="O55" s="7" t="n"/>
-      <c r="P55" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  generate_telemetry_report FinOps + telemetry summary</t>
-        </is>
-      </c>
+      <c r="P55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="O56" s="7" t="n"/>
-      <c r="P56" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  rotate_logs               Archive and purge logs</t>
-        </is>
-      </c>
+      <c r="P56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="O57" s="7" t="n"/>
-      <c r="P57" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Render &amp; FinOps</t>
-        </is>
-      </c>
+      <c r="P57" s="10" t="n"/>
     </row>
     <row r="58">
       <c r="O58" s="7" t="n"/>
-      <c r="P58" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  execute_render_pipeline   Fire TTS+image+FFmpeg</t>
-        </is>
-      </c>
+      <c r="P58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="O59" s="7" t="n"/>
-      <c r="P59" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  estimate_manifest_cost    USD cost estimate (pre-fire)</t>
-        </is>
-      </c>
+      <c r="P59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="O60" s="7" t="n"/>
-      <c r="P60" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Orchestration</t>
-        </is>
-      </c>
+      <c r="P60" s="10" t="n"/>
     </row>
     <row r="61">
       <c r="O61" s="7" t="n"/>
-      <c r="P61" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  mint_agent                Create agent definition</t>
-        </is>
-      </c>
+      <c r="P61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="O62" s="7" t="n"/>
-      <c r="P62" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  build_topology            Build topology CSV</t>
-        </is>
-      </c>
+      <c r="P62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="O63" s="7" t="n"/>
-      <c r="P63" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  link_projects             Synaptic Bridge two silos</t>
-        </is>
-      </c>
+      <c r="P63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="O64" s="7" t="n"/>
-      <c r="P64" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ignite_swarm              Inject payload + start swarm</t>
-        </is>
-      </c>
+      <c r="P64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="O65" s="7" t="n"/>
-      <c r="P65" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  initialize_workspace      Provision 6-tier silo</t>
-        </is>
-      </c>
+      <c r="P65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="O66" s="7" t="n"/>
-      <c r="P66" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  switch_workspace          Change active project</t>
-        </is>
-      </c>
+      <c r="P66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="O67" s="7" t="n"/>
-      <c r="P67" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  request_elevation         PIN-gate for privileged ops</t>
-        </is>
-      </c>
+      <c r="P67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="O68" s="7" t="n"/>
-      <c r="P68" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  promote_topology_to_library  Save topology to library</t>
-        </is>
-      </c>
+      <c r="P68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="O69" s="7" t="n"/>
-      <c r="P69" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  recall_topology           Load named topology</t>
-        </is>
-      </c>
+      <c r="P69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="O70" s="7" t="n"/>
-      <c r="P70" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  design_swarm              Agentic swarm design</t>
-        </is>
-      </c>
+      <c r="P70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="O71" s="7" t="n"/>
-      <c r="P71" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  run_swarm                 Execute swarm worker loop</t>
-        </is>
-      </c>
+      <c r="P71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="O72" s="7" t="n"/>
-      <c r="P72" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  create_persona_card       Generate agent persona</t>
-        </is>
-      </c>
+      <c r="P72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="O73" s="7" t="n"/>
-      <c r="P73" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sync &amp; Utilities</t>
-        </is>
-      </c>
+      <c r="P73" s="10" t="n"/>
     </row>
     <row r="74">
       <c r="O74" s="7" t="n"/>
-      <c r="P74" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  export_project_nugget     Export nugget to Drive</t>
-        </is>
-      </c>
+      <c r="P74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="O75" s="7" t="n"/>
-      <c r="P75" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  import_project_nuggets    Import nuggets from Drive</t>
-        </is>
-      </c>
+      <c r="P75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="O76" s="7" t="n"/>
-      <c r="P76" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  list_project_nuggets      List Drive nuggets</t>
-        </is>
-      </c>
+      <c r="P76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="O77" s="7" t="n"/>
-      <c r="P77" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ensure_project_workbook   Guarantee Session.xlsx exists</t>
-        </is>
-      </c>
+      <c r="P77" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2989,10 +3050,10 @@
   </mergeCells>
   <dataValidations count="7">
     <dataValidation sqref="A3:A200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="New Agent Name" error="This agent is not in the existing roster. Click YES to keep this name — the agent will be defined by the row settings and minted into the project on successful workbook execution. Click NO to pick from the dropdown instead." type="list" errorStyle="warning">
-      <formula1>'_AGENTS'!$A$1:$A$1</formula1>
+      <formula1>'_AGENTS'!$A$1:$A$26</formula1>
     </dataValidation>
     <dataValidation sqref="B3:B200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Choose a value from the dropdown list." type="list" errorStyle="stop">
-      <formula1>'_MODELS'!$A$1:$A$54</formula1>
+      <formula1>'_MODELS'!$A$1:$A$55</formula1>
     </dataValidation>
     <dataValidation sqref="C3:C200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Choose a value from the dropdown list." type="list" errorStyle="stop">
       <formula1>"Researcher,Writer,Synthesiser,Director,Critic,Extractor,Verifier,Renderer,Archivist,Router"</formula1>
@@ -3020,7 +3081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3033,8 +3094,8 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="35" customWidth="1" min="10" max="10"/>
-    <col width="1.5" customWidth="1" min="11" max="11"/>
-    <col width="58" customWidth="1" min="12" max="12"/>
+    <col width="1.5" customWidth="1" min="13" max="13"/>
+    <col width="58" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -3095,391 +3156,249 @@
           <t>ARTIFACT_PATH</t>
         </is>
       </c>
-      <c r="K2" s="7" t="n"/>
-      <c r="L2" s="8" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>DIALOGUE_PARTNER</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>DIALOGUE_ROUNDS</t>
+        </is>
+      </c>
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="8" t="inlineStr">
         <is>
           <t>📖  TOPOLOGY — REFERENCE</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>NODE_01</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>MyAgent</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>START_CONVO</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MemoryReporter</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>STOP</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr"/>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>Write a brief from the payload.</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr"/>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>STOP</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr"/>
-      <c r="K3" s="7" t="n"/>
-      <c r="L3" s="9" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>SourceReader|Synthesizer</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="n"/>
+      <c r="N3" s="9" t="n"/>
     </row>
     <row r="4">
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="10" t="inlineStr">
-        <is>
-          <t>NODE_ID  (col A)</t>
-        </is>
-      </c>
+      <c r="M4" s="7" t="n"/>
+      <c r="N4" s="10" t="n"/>
     </row>
     <row r="5">
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="12" t="inlineStr">
-        <is>
-          <t>Unique name. Convention: ROLE_PURPOSE</t>
-        </is>
-      </c>
+      <c r="M5" s="7" t="n"/>
+      <c r="N5" s="12" t="n"/>
     </row>
     <row r="6">
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="12" t="inlineStr">
-        <is>
-          <t>Example: RESEARCHER_OSINT, CRITIC_QUALITY</t>
-        </is>
-      </c>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="12" t="n"/>
     </row>
     <row r="7">
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="9" t="inlineStr"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="10" t="inlineStr">
-        <is>
-          <t>NEXT_NODE  (col C) — terminal keywords</t>
-        </is>
-      </c>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="10" t="n"/>
     </row>
     <row r="9">
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  STOP    Clean termination  (primary keyword)</t>
-        </is>
-      </c>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  DONE    Alias for STOP</t>
-        </is>
-      </c>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FAILED  Error termination path</t>
-        </is>
-      </c>
+      <c r="M11" s="7" t="n"/>
+      <c r="N11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="K12" s="7" t="n"/>
-      <c r="L12" s="9" t="inlineStr"/>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="9" t="n"/>
     </row>
     <row r="13">
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="10" t="inlineStr">
-        <is>
-          <t>WAIT_FOR  (col G) — fan-in gate</t>
-        </is>
-      </c>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="K14" s="7" t="n"/>
-      <c r="L14" s="12" t="inlineStr">
-        <is>
-          <t>Comma-separated NODE_IDs this node waits for.</t>
-        </is>
-      </c>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="12" t="n"/>
     </row>
     <row r="15">
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="12" t="inlineStr">
-        <is>
-          <t>Fires only after ALL listed nodes complete.</t>
-        </is>
-      </c>
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="12" t="n"/>
     </row>
     <row r="16">
-      <c r="K16" s="7" t="n"/>
-      <c r="L16" s="12" t="inlineStr">
-        <is>
-          <t>Use for Synthesiser nodes merging parallel paths.</t>
-        </is>
-      </c>
+      <c r="M16" s="7" t="n"/>
+      <c r="N16" s="12" t="n"/>
     </row>
     <row r="17">
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="12" t="inlineStr">
-        <is>
-          <t>Example: WAIT_FOR = OSINT_GOOGLE,OSINT_BRAVE</t>
-        </is>
-      </c>
+      <c r="M17" s="7" t="n"/>
+      <c r="N17" s="12" t="n"/>
     </row>
     <row r="18">
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="9" t="inlineStr"/>
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="9" t="n"/>
     </row>
     <row r="19">
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="10" t="inlineStr">
-        <is>
-          <t>FAILURE_TARGET  (col H) — circuit breaker</t>
-        </is>
-      </c>
+      <c r="M19" s="7" t="n"/>
+      <c r="N19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="12" t="inlineStr">
-        <is>
-          <t>Route here if node hits error or MAX_RECURSION</t>
-        </is>
-      </c>
+      <c r="M20" s="7" t="n"/>
+      <c r="N20" s="12" t="n"/>
     </row>
     <row r="21">
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="12" t="inlineStr">
-        <is>
-          <t>expires. Typically STOP or DONE.</t>
-        </is>
-      </c>
+      <c r="M21" s="7" t="n"/>
+      <c r="N21" s="12" t="n"/>
     </row>
     <row r="22">
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="9" t="inlineStr"/>
+      <c r="M22" s="7" t="n"/>
+      <c r="N22" s="9" t="n"/>
     </row>
     <row r="23">
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="10" t="inlineStr">
-        <is>
-          <t>MAX_RECURSION  (col I)</t>
-        </is>
-      </c>
+      <c r="M23" s="7" t="n"/>
+      <c r="N23" s="10" t="n"/>
     </row>
     <row r="24">
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="12" t="inlineStr">
-        <is>
-          <t>SQLite queue-level counter. Not agent reasoning.</t>
-        </is>
-      </c>
+      <c r="M24" s="7" t="n"/>
+      <c r="N24" s="12" t="n"/>
     </row>
     <row r="25">
-      <c r="K25" s="7" t="n"/>
-      <c r="L25" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0  Executes once. Re-entry → FAILURE_TARGET.</t>
-        </is>
-      </c>
+      <c r="M25" s="7" t="n"/>
+      <c r="N25" s="11" t="n"/>
     </row>
     <row r="26">
-      <c r="K26" s="7" t="n"/>
-      <c r="L26" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  3  Initial + 3 re-entries = 4 total executions.</t>
-        </is>
-      </c>
+      <c r="M26" s="7" t="n"/>
+      <c r="N26" s="11" t="n"/>
     </row>
     <row r="27">
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="12" t="inlineStr">
-        <is>
-          <t>Critic loop: Critic MAX=3, Writer MAX=0.</t>
-        </is>
-      </c>
+      <c r="M27" s="7" t="n"/>
+      <c r="N27" s="12" t="n"/>
     </row>
     <row r="28">
-      <c r="K28" s="7" t="n"/>
-      <c r="L28" s="9" t="inlineStr"/>
+      <c r="M28" s="7" t="n"/>
+      <c r="N28" s="9" t="n"/>
     </row>
     <row r="29">
-      <c r="K29" s="7" t="n"/>
-      <c r="L29" s="10" t="inlineStr">
-        <is>
-          <t>─── PATTERNS ─────────────────────────────────────────</t>
-        </is>
-      </c>
+      <c r="M29" s="7" t="n"/>
+      <c r="N29" s="10" t="n"/>
     </row>
     <row r="30">
-      <c r="K30" s="7" t="n"/>
-      <c r="L30" s="9" t="inlineStr"/>
+      <c r="M30" s="7" t="n"/>
+      <c r="N30" s="9" t="n"/>
     </row>
     <row r="31">
-      <c r="K31" s="7" t="n"/>
-      <c r="L31" s="10" t="inlineStr">
-        <is>
-          <t>CRITIC LOOP</t>
-        </is>
-      </c>
+      <c r="M31" s="7" t="n"/>
+      <c r="N31" s="10" t="n"/>
     </row>
     <row r="32">
-      <c r="K32" s="7" t="n"/>
-      <c r="L32" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  WRITER  Writer   NEXT:CRITIC   MAX_REC:0</t>
-        </is>
-      </c>
+      <c r="M32" s="7" t="n"/>
+      <c r="N32" s="11" t="n"/>
     </row>
     <row r="33">
-      <c r="K33" s="7" t="n"/>
-      <c r="L33" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CRITIC  Critic   NEXT:STOP     MAX_REC:3</t>
-        </is>
-      </c>
+      <c r="M33" s="7" t="n"/>
+      <c r="N33" s="11" t="n"/>
     </row>
     <row r="34">
-      <c r="K34" s="7" t="n"/>
-      <c r="L34" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Critic instruction: Score 1-10. If ≥8: ROUTE:STOP.</t>
-        </is>
-      </c>
+      <c r="M34" s="7" t="n"/>
+      <c r="N34" s="12" t="n"/>
     </row>
     <row r="35">
-      <c r="K35" s="7" t="n"/>
-      <c r="L35" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  If &lt;8: ROUTE:WRITER with revision notes.</t>
-        </is>
-      </c>
+      <c r="M35" s="7" t="n"/>
+      <c r="N35" s="12" t="n"/>
     </row>
     <row r="36">
-      <c r="K36" s="7" t="n"/>
-      <c r="L36" s="9" t="inlineStr"/>
+      <c r="M36" s="7" t="n"/>
+      <c r="N36" s="9" t="n"/>
     </row>
     <row r="37">
-      <c r="K37" s="7" t="n"/>
-      <c r="L37" s="10" t="inlineStr">
-        <is>
-          <t>FAN-OUT / FAN-IN</t>
-        </is>
-      </c>
+      <c r="M37" s="7" t="n"/>
+      <c r="N37" s="10" t="n"/>
     </row>
     <row r="38">
-      <c r="K38" s="7" t="n"/>
-      <c r="L38" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FORK    Director    NEXT:PATH_A</t>
-        </is>
-      </c>
+      <c r="M38" s="7" t="n"/>
+      <c r="N38" s="11" t="n"/>
     </row>
     <row r="39">
-      <c r="K39" s="7" t="n"/>
-      <c r="L39" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PATH_A  Researcher  NEXT:MERGER</t>
-        </is>
-      </c>
+      <c r="M39" s="7" t="n"/>
+      <c r="N39" s="11" t="n"/>
     </row>
     <row r="40">
-      <c r="K40" s="7" t="n"/>
-      <c r="L40" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PATH_B  Researcher  NEXT:MERGER</t>
-        </is>
-      </c>
+      <c r="M40" s="7" t="n"/>
+      <c r="N40" s="11" t="n"/>
     </row>
     <row r="41">
-      <c r="K41" s="7" t="n"/>
-      <c r="L41" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MERGER  Synthesiser NEXT:STOP  WAIT_FOR:PATH_A,PATH_B</t>
-        </is>
-      </c>
+      <c r="M41" s="7" t="n"/>
+      <c r="N41" s="11" t="n"/>
     </row>
     <row r="42">
-      <c r="K42" s="7" t="n"/>
-      <c r="L42" s="9" t="inlineStr"/>
+      <c r="M42" s="7" t="n"/>
+      <c r="N42" s="9" t="n"/>
     </row>
     <row r="43">
-      <c r="K43" s="7" t="n"/>
-      <c r="L43" s="10" t="inlineStr">
-        <is>
-          <t>HYBRID-SYNTHESIS OSINT</t>
-        </is>
-      </c>
+      <c r="M43" s="7" t="n"/>
+      <c r="N43" s="10" t="n"/>
     </row>
     <row r="44">
-      <c r="K44" s="7" t="n"/>
-      <c r="L44" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  OSINT_G  Researcher NEXT:DEDUP GROUNDING:Google</t>
-        </is>
-      </c>
+      <c r="M44" s="7" t="n"/>
+      <c r="N44" s="11" t="n"/>
     </row>
     <row r="45">
-      <c r="K45" s="7" t="n"/>
-      <c r="L45" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  OSINT_B  Researcher NEXT:DEDUP GROUNDING:Brave</t>
-        </is>
-      </c>
+      <c r="M45" s="7" t="n"/>
+      <c r="N45" s="11" t="n"/>
     </row>
     <row r="46">
-      <c r="K46" s="7" t="n"/>
-      <c r="L46" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  DEDUP    Extractor  NEXT:SYNTH WAIT_FOR:OSINT_G,OSINT_B</t>
-        </is>
-      </c>
+      <c r="M46" s="7" t="n"/>
+      <c r="N46" s="11" t="n"/>
     </row>
     <row r="47">
-      <c r="K47" s="7" t="n"/>
-      <c r="L47" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SYNTH    Synthesiser NEXT:STOP</t>
-        </is>
-      </c>
+      <c r="M47" s="7" t="n"/>
+      <c r="N47" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="B3:B50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Agent Not in Roster" error="This agent is not in the current project roster. Click YES to use this name - the agent must be defined in the AGENTS sheet and will be minted on first execution." type="list" errorStyle="warning">
-      <formula1>"MyAgent"</formula1>
+      <formula1>"MemoryReporter,SourceReader,Synthesizer"</formula1>
     </dataValidation>
     <dataValidation sqref="C3:C50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Choose a value from the dropdown list." type="list" errorStyle="stop">
-      <formula1>"NODE_01,STOP,DONE,FAILED"</formula1>
+      <formula1>"START_CONVO,STOP,DONE,FAILED"</formula1>
     </dataValidation>
     <dataValidation sqref="D3:D50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Choose a value from the dropdown list." type="list" errorStyle="stop">
-      <formula1>'_MODELS'!$A$1:$A$54</formula1>
+      <formula1>'_MODELS'!$A$1:$A$55</formula1>
     </dataValidation>
     <dataValidation sqref="H3:H50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Choose a value from the dropdown list." type="list" errorStyle="stop">
-      <formula1>"NODE_01,STOP,DONE,FAILED"</formula1>
+      <formula1>"START_CONVO,STOP,DONE,FAILED"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3565,12 +3484,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>META_TEST</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>cloud</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>START_CONVO</t>
         </is>
       </c>
       <c r="I3" s="7" t="n"/>
@@ -4006,102 +3930,102 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>PROJECT_DEFINITION</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
       </c>
-      <c r="C3" s="15" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D3" s="15" t="n">
+      <c r="D3" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>AGENTS</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="14" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>TOPOLOGY</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="n">
         <v>0.0009</v>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>TOPOLOGY</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>SWARM_REQUEST</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D5" s="15" t="n">
-        <v>0.0009</v>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>SWARM_REQUEST</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>START_NODE missing; No payload (PAYLOAD_TEXT or PAYLOAD_PATH) — swarm will not run</t>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>No payload (PAYLOAD_TEXT or PAYLOAD_PATH) — swarm will not run</t>
         </is>
       </c>
     </row>

</xml_diff>